<commit_message>
progress: 30 village workbooks (randomwalk-TRX50-WS 2026-10-09T15:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chinnasholianpakkam_13.412594_80.14907.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chinnasholianpakkam_13.412594_80.14907.xlsx
@@ -806,11 +806,6 @@
           <t>39</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10, 1A, 1B, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C, 7A1, 7A2, 7A3, 7A4, 7B1, 7B2, 7B3, 8A, 8B, 9</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -818,11 +813,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C1, 1C2A, 1C2B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -830,11 +820,6 @@
           <t>40</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2A3, 2B, 3, 4A, 4B, 5</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -842,11 +827,6 @@
           <t>41</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>1, 2A1, 2A2, 2B, 3A1, 3A2, 3A3, 3B1, 3B2, 4A, 4B, 4C, 4D, 4E, 5</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -854,11 +834,6 @@
           <t>42</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -866,11 +841,6 @@
           <t>43</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -878,11 +848,6 @@
           <t>44</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -890,11 +855,6 @@
           <t>45</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B1, 3B2, 3B3, 3B4, 3B5, 4A1, 4A2, 4A3, 4A4, 4A5, 4B1, 4B2, 4B3, 4B4, 4B5, 5</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -902,11 +862,6 @@
           <t>46</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4A1, 4A2, 4A3, 4B, 5A, 5B, 6A, 6B, 7A1A, 7A1B, 7A1C, 7A2, 7B, 8A1, 8A2, 8B, 8C, 8D, 9</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -914,11 +869,6 @@
           <t>47</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -926,11 +876,6 @@
           <t>48</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>1A, 1B, 1C, 1D, 1E, 1F, 2</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -938,11 +883,6 @@
           <t>49</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 5D, 6A, 6B, 6C, 7, 8A, 8B, 8C, 8D, 8E</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -950,11 +890,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>1A, 1B1, 1B2, 1C, 2, 3</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -962,11 +897,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -974,11 +904,6 @@
           <t>500</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -986,11 +911,6 @@
           <t>51</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -998,11 +918,6 @@
           <t>52</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1010,11 +925,6 @@
           <t>53</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1022,11 +932,6 @@
           <t>54</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1034,11 +939,6 @@
           <t>55</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1046,11 +946,6 @@
           <t>56</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>1A, 1B, 2, 3, 4, 5A1, 5A2, 5B, 6A1, 6A2, 6B, 7A, 7B, 8</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1058,11 +953,6 @@
           <t>57</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1070,11 +960,6 @@
           <t>58</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1082,11 +967,6 @@
           <t>59</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1094,11 +974,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4A, 4B, 5, 6</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1106,11 +981,6 @@
           <t>60</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1118,11 +988,6 @@
           <t>61</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1130,11 +995,6 @@
           <t>62</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1142,11 +1002,6 @@
           <t>63</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1154,11 +1009,6 @@
           <t>64</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1166,11 +1016,6 @@
           <t>65</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1178,11 +1023,6 @@
           <t>66</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1190,11 +1030,6 @@
           <t>67</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1202,11 +1037,6 @@
           <t>68</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1214,11 +1044,6 @@
           <t>69</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1226,11 +1051,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>1, 2</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1238,11 +1058,6 @@
           <t>70</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1, 1B, 2A, 2B, 3A, 3B, 3C, 4, 5A, 5B, 6A, 6B, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1250,11 +1065,6 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1262,11 +1072,6 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1274,11 +1079,6 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3A, 3B1, 3B2, 4A1A, 4A1B, 4A2, 4A3, 4B, 5A, 5B1, 5B2, 5B3</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1286,11 +1086,6 @@
           <t>74</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1298,21 +1093,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
           <t>9</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>1A, 2A, 2B, 3, 4A, 4B, 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 32 village workbooks (randomwalk-TRX50-WS 2026-10-09T15:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Chinnasholianpakkam_13.412594_80.14907.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Chinnasholianpakkam_13.412594_80.14907.xlsx
@@ -806,6 +806,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B, 2, 3, 4A, 4B, 5A, 5B, 5C, 6A, 6B, 6C, 7A1, 7A2, 7A3, 7A4, 7B1, 7B2, 7B3, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -813,6 +818,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2A, 1C2B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -820,6 +830,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -827,6 +842,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3A1, 3A2, 3A3, 3B1, 3B2, 4A, 4B, 4C, 4D, 4E, 5</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -834,6 +854,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -841,6 +866,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -848,6 +878,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 2</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -855,6 +890,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 3B3, 3B4, 3B5, 4A1, 4A2, 4A3, 4A4, 4A5, 4B1, 4B2, 4B3, 4B4, 4B5, 5</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -862,6 +902,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A1, 4A2, 4A3, 4B, 5A, 5B, 6A, 6B, 7A1A, 7A1B, 7A1C, 7A2, 7B, 8A1, 8A2, 8B, 8C, 8D, 9</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -869,6 +914,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -876,6 +926,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -883,6 +938,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 5D, 6A, 6B, 6C, 7, 8A, 8B, 8C, 8D, 8E</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -890,6 +950,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -897,6 +962,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -904,6 +974,11 @@
           <t>500</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -911,6 +986,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -918,6 +998,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -925,6 +1010,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -932,6 +1022,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -939,6 +1034,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -946,6 +1046,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A1, 5A2, 5B, 6A1, 6A2, 6B, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -953,6 +1058,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -960,6 +1070,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -967,6 +1082,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -974,6 +1094,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -981,6 +1106,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -988,6 +1118,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -995,6 +1130,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1002,6 +1142,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1009,6 +1154,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1016,6 +1166,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1023,6 +1178,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1030,6 +1190,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4A, 4B, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1037,6 +1202,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1044,6 +1214,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1051,6 +1226,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1058,6 +1238,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 1B, 2A, 2B, 3A, 3B, 3C, 4, 5A, 5B, 6A, 6B, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1065,6 +1250,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1072,6 +1262,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1079,6 +1274,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B, 2A, 2B, 3A, 3B1, 3B2, 4A1A, 4A1B, 4A2, 4A3, 4B, 5A, 5B1, 5B2, 5B3</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1086,6 +1286,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1093,11 +1298,21 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
           <t>9</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1A, 2A, 2B, 3, 4A, 4B, 5</t>
         </is>
       </c>
     </row>

</xml_diff>